<commit_message>
feat: Excel'de yorum tarihi (mail zamanı), boş değer temizliği
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/cevaplar/yorum-cevaplari.xlsx
+++ b/agent/cevaplar/yorum-cevaplari.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Taslak tarihi</t>
+          <t>Yorum tarihi</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bugün</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,7 +511,11 @@
       <c r="D2" t="n">
         <v>5</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Vallahi ben bu kadar beklemezdim . tesadüfen Süleymaniye camiden indim . İyiki oraya inmiş im kokoreç güzel değil süper arkadaşa sade istedim bana unutmayacağım bı lezzzet sundu. Kralsinsiniz çok yakında oradayım her istanbul turunda ziyaret listemde artik</t>
@@ -548,7 +552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bugün</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -559,7 +563,11 @@
       <c r="D3" t="n">
         <v>3</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Sakin bir saatte kokoreç tercih ettik. İzmir usulü kokoreç istedim üç çeyrek olarak. Ne yazık ki bir egeli olarak İzmir kokoreçi hakkıyla yapan bir mekan bulmakta oldukça zorlanıyorum. İzmir kokoreç dediğin iri kıyım ve sulu sulu olur. Genelde hep kokoreçi kurutup ekmeğin arasına koyup getiriyorlar. Burasıda öyleydi ne yazık ki. Lezzetsiz bir mekan diyemem ama İzmir kokoreç sever birisiyseniz pek tatmin etmeyebilir.</t>
@@ -596,7 +604,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bugün</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -607,7 +615,11 @@
       <c r="D4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>İzmir usulünü tavsiye etmem sirkülasyon çok olduğu için düzgün pişirilmemişti, ekmeğin içinin kızarması ve kokoreç halkalarının son pişirmesinin parçalanmadan yapılması ve ekmeğin içinde kesilmesi gerekir. Tezgahın büyütülmesi gerekir yetmiyor, yoğunlukta kalite hızlı düşüyor,normalde iyi ve eski bir kokoreççi</t>
@@ -644,7 +656,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bugün</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -655,7 +667,11 @@
       <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>1 defa ziyaret etmiştim. Balık ekmek yedikten sonra bir de üstüne kokoreç yiyeyim diyip uğradım. Kokoreç güzeldi, beğendim. İçerisi ufak ama yer buldum, hızlı geldi, fiyatı da makuldü. Memnun kaldım.</t>
@@ -692,7 +708,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bugün</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -703,7 +719,11 @@
       <c r="D6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>“Uzun zamandır böyle lezzetli kokoreç yememiştim. Malzeme kaliteli, kokusu bile iştah açıyor. Salaş ama samimi bir ortamı var, tam kokoreççinin olması gerektiği gibi.”</t>
@@ -740,7 +760,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -796,7 +816,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bugün</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>